<commit_message>
data: issues 001, 002, 003, 004, 005, 006, 007
</commit_message>
<xml_diff>
--- a/001/xy_001_data.xlsx
+++ b/001/xy_001_data.xlsx
@@ -588,7 +588,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>25/09/2026 01:04</t>
+          <t>25/09/2026 01:16</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>25/09/2026 01:04</t>
+          <t>25/09/2026 01:16</t>
         </is>
       </c>
     </row>

</xml_diff>